<commit_message>
export image into pdf
</commit_message>
<xml_diff>
--- a/public/data/np_geostory_2025-09-30.xlsx
+++ b/public/data/np_geostory_2025-09-30.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\Documents\other-prj\geospatial-stories\gv-ssr-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7AD178-3C9C-41C0-84E4-3B283E71E40A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAA9308-73FC-4CC5-8B08-4482220EBD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="127">
   <si>
     <t>geostory_id</t>
   </si>
@@ -193,9 +193,6 @@
   </si>
   <si>
     <t>"Scenario 3: Blue Development (BD) " + scenarioSoS_bd$general_description</t>
-  </si>
-  <si>
-    <t>img:https://drive.google.com/file/d/16uG1eZW_UHT_IzqnAZ3imh8phOQWX386/view?usp=drive_link; alt:"immagine di copertina in cui si vede una barca a vela che veleggia nel mare"</t>
   </si>
   <si>
     <t>main_background</t>
@@ -413,9 +410,6 @@
     <t>Regolamentazione e sicurezza</t>
   </si>
   <si>
-    <t>forse non necessario perché già presente per temi in foglio di scenario</t>
-  </si>
-  <si>
     <t>Lo scenario è definito da una narrativa sintetica che ne esprime la visione, da un orizzonte temporale di riferimento e da un elenco di settori principali e secondari.</t>
   </si>
   <si>
@@ -424,12 +418,28 @@
   <si>
     <t>"Stato giuridico dell’area di studio Lo scenario assume che sia istituita la zona economica esclusiva con limiti esterni corrispondenti a quelli indicati nel Piano MSP approvato."</t>
   </si>
+  <si>
+    <t>unknow:https://drive.google.com/file/d/16uG1eZW_UHT_IzqnAZ3imh8phOQWX386/view?usp=drive_link; alt:"immagine di copertina in cui si vede una barca a vela che veleggia nel mare"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">img: https://design-earth.org/files/gimgs/193_056B8804.jpg
+  </t>
+  </si>
+  <si>
+    <t>img:https://metropolismag.com/wp-content/uploads/2021/07/DE_PacificAquarium_03.jpg</t>
+  </si>
+  <si>
+    <t>img: https://metropolismag.com/wp-content/uploads/2021/07/DE_PacificAquarium_01.jpg</t>
+  </si>
+  <si>
+    <t>img:https://metropolismag.com/wp-content/uploads/2021/07/DE_Of-Oil-and-Ice_01.jpg</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -531,6 +541,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -623,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -680,9 +705,6 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -708,6 +730,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -29299,7 +29325,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AE25"/>
+  <dimension ref="A1:AE36"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.28515625" customWidth="1"/>
@@ -29399,22 +29425,22 @@
       <c r="H2" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="J2" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="K2" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="L2" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="M2" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M2" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N2" s="21"/>
+      <c r="N2" s="20"/>
       <c r="O2" s="16"/>
       <c r="P2" s="16"/>
       <c r="Q2" s="16"/>
@@ -29438,41 +29464,41 @@
         <v>2</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="G3" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="H3" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="L3" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H3" s="16" t="s">
-        <v>121</v>
+      <c r="M3" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="I3" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K3" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L3" s="16" t="s">
+      <c r="N3" s="20" t="s">
         <v>63</v>
-      </c>
-      <c r="M3" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N3" s="21" t="s">
-        <v>64</v>
       </c>
       <c r="O3" s="16"/>
       <c r="P3" s="16"/>
@@ -29497,38 +29523,38 @@
         <v>3</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C4" s="17"/>
       <c r="D4" s="19"/>
       <c r="E4" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="22" t="s">
-        <v>62</v>
+      <c r="I4" s="16" t="s">
+        <v>124</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="J4" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="I4" s="16" t="s">
-        <v>55</v>
+      <c r="M4" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="J4" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K4" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L4" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="M4" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N4" s="21"/>
+      <c r="N4" s="20"/>
       <c r="O4" s="16"/>
       <c r="P4" s="16"/>
       <c r="Q4" s="16"/>
@@ -29552,38 +29578,38 @@
         <v>4</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="19"/>
       <c r="E5" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="G5" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="L5" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="22" t="s">
-        <v>62</v>
+      <c r="M5" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="H5" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="I5" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L5" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="M5" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N5" s="21"/>
+      <c r="N5" s="20"/>
       <c r="O5" s="16"/>
       <c r="P5" s="16"/>
       <c r="Q5" s="16"/>
@@ -29607,41 +29633,41 @@
         <v>5</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="G6" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="G6" s="22" t="s">
-        <v>62</v>
+      <c r="I6" s="16" t="s">
+        <v>126</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="J6" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="I6" s="16" t="s">
-        <v>55</v>
+      <c r="M6" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="J6" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K6" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L6" s="16" t="s">
+      <c r="N6" s="23" t="s">
         <v>75</v>
-      </c>
-      <c r="M6" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N6" s="24" t="s">
-        <v>76</v>
       </c>
       <c r="O6" s="16"/>
       <c r="P6" s="16"/>
@@ -29666,41 +29692,41 @@
         <v>6</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D7" s="19"/>
       <c r="E7" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="G7" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="G7" s="22" t="s">
-        <v>62</v>
+      <c r="I7" t="s">
+        <v>54</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="J7" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="I7" s="16" t="s">
-        <v>55</v>
+      <c r="M7" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K7" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L7" s="16" t="s">
+      <c r="N7" s="23" t="s">
         <v>80</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N7" s="24" t="s">
-        <v>81</v>
       </c>
       <c r="O7" s="16"/>
       <c r="P7" s="16"/>
@@ -29725,41 +29751,41 @@
         <v>7</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D8" s="19"/>
       <c r="E8" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="G8" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="I8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="G8" s="22" t="s">
-        <v>62</v>
+      <c r="M8" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="H8" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="I8" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K8" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="L8" s="16" t="s">
+      <c r="N8" s="23" t="s">
         <v>84</v>
-      </c>
-      <c r="M8" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N8" s="24" t="s">
-        <v>85</v>
       </c>
       <c r="O8" s="16"/>
       <c r="P8" s="16"/>
@@ -29784,41 +29810,41 @@
         <v>8</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D9" s="19"/>
       <c r="E9" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="G9" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="H9" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="I9" t="s">
         <v>91</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="J9" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K9" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="J9" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K9" s="17" t="s">
+      <c r="L9" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="L9" s="25" t="s">
+      <c r="M9" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N9" s="25" t="s">
         <v>94</v>
-      </c>
-      <c r="M9" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N9" s="26" t="s">
-        <v>95</v>
       </c>
       <c r="O9" s="16"/>
       <c r="P9" s="16"/>
@@ -29843,41 +29869,41 @@
         <v>9</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D10" s="19"/>
       <c r="E10" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="G10" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="G10" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="H10" s="27" t="s">
+      <c r="I10" t="s">
         <v>98</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="J10" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="K10" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="J10" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K10" s="17" t="s">
+      <c r="L10" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="L10" s="16" t="s">
+      <c r="M10" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N10" s="23" t="s">
         <v>101</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N10" s="24" t="s">
-        <v>102</v>
       </c>
       <c r="O10" s="16"/>
       <c r="P10" s="16"/>
@@ -29902,37 +29928,37 @@
         <v>10</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D11" s="19"/>
       <c r="E11" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F11" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="G11" s="22" t="s">
-        <v>62</v>
+      <c r="J11" s="17" t="s">
+        <v>54</v>
       </c>
-      <c r="H11" s="27" t="s">
+      <c r="K11" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="J11" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K11" s="17" t="s">
+      <c r="L11" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="L11" s="16" t="s">
-        <v>106</v>
+      <c r="M11" s="16" t="s">
+        <v>56</v>
       </c>
-      <c r="M11" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="N11" s="21"/>
+      <c r="N11" s="20"/>
       <c r="O11" s="16"/>
       <c r="P11" s="16"/>
       <c r="Q11" s="16"/>
@@ -29956,35 +29982,35 @@
         <v>11</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F12" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="G12" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>108</v>
-      </c>
       <c r="J12" s="17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K12" s="17"/>
       <c r="L12" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
-      <c r="N12" s="21"/>
+      <c r="N12" s="20"/>
       <c r="O12" s="16"/>
       <c r="P12" s="16"/>
       <c r="Q12" s="16"/>
@@ -30008,38 +30034,38 @@
         <v>12</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F13" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H13" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="G13" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="H13" s="27" t="s">
+      <c r="I13" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="I13" s="27" t="s">
-        <v>112</v>
-      </c>
       <c r="J13" s="17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K13" s="17"/>
       <c r="L13" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
-      <c r="N13" s="21"/>
+      <c r="N13" s="20"/>
       <c r="O13" s="16"/>
       <c r="P13" s="16"/>
       <c r="Q13" s="16"/>
@@ -30063,35 +30089,35 @@
         <v>13</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D14" s="19"/>
       <c r="E14" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F14" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H14" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="G14" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>115</v>
-      </c>
       <c r="J14" s="17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K14" s="17"/>
       <c r="L14" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
-      <c r="N14" s="21"/>
+      <c r="N14" s="20"/>
       <c r="O14" s="16"/>
       <c r="P14" s="16"/>
       <c r="Q14" s="16"/>
@@ -30115,35 +30141,35 @@
         <v>14</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D15" s="19"/>
       <c r="E15" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F15" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="G15" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="H15" s="27" t="s">
-        <v>118</v>
-      </c>
       <c r="J15" s="17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K15" s="17"/>
       <c r="L15" s="16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M15" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
-      <c r="N15" s="21"/>
+      <c r="N15" s="20"/>
       <c r="O15" s="16"/>
       <c r="P15" s="16"/>
       <c r="Q15" s="16"/>
@@ -30176,7 +30202,7 @@
       <c r="K16" s="17"/>
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
-      <c r="N16" s="21"/>
+      <c r="N16" s="20"/>
       <c r="O16" s="16"/>
       <c r="P16" s="16"/>
       <c r="Q16" s="16"/>
@@ -30209,7 +30235,7 @@
       <c r="K17" s="17"/>
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
-      <c r="N17" s="21"/>
+      <c r="N17" s="20"/>
       <c r="O17" s="16"/>
       <c r="P17" s="16"/>
       <c r="Q17" s="16"/>
@@ -30242,7 +30268,7 @@
       <c r="K18" s="17"/>
       <c r="L18" s="16"/>
       <c r="M18" s="16"/>
-      <c r="N18" s="21"/>
+      <c r="N18" s="20"/>
       <c r="O18" s="16"/>
       <c r="P18" s="16"/>
       <c r="Q18" s="16"/>
@@ -30275,7 +30301,7 @@
       <c r="K19" s="17"/>
       <c r="L19" s="16"/>
       <c r="M19" s="16"/>
-      <c r="N19" s="21"/>
+      <c r="N19" s="20"/>
       <c r="O19" s="16"/>
       <c r="P19" s="16"/>
       <c r="Q19" s="16"/>
@@ -30308,7 +30334,7 @@
       <c r="K20" s="17"/>
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
-      <c r="N20" s="21"/>
+      <c r="N20" s="20"/>
       <c r="O20" s="16"/>
       <c r="P20" s="16"/>
       <c r="Q20" s="16"/>
@@ -30341,7 +30367,7 @@
       <c r="K21" s="17"/>
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
-      <c r="N21" s="21"/>
+      <c r="N21" s="20"/>
       <c r="O21" s="16"/>
       <c r="P21" s="16"/>
       <c r="Q21" s="16"/>
@@ -30374,7 +30400,7 @@
       <c r="K22" s="17"/>
       <c r="L22" s="16"/>
       <c r="M22" s="16"/>
-      <c r="N22" s="21"/>
+      <c r="N22" s="20"/>
       <c r="O22" s="16"/>
       <c r="P22" s="16"/>
       <c r="Q22" s="16"/>
@@ -30407,7 +30433,7 @@
       <c r="K23" s="17"/>
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
-      <c r="N23" s="21"/>
+      <c r="N23" s="20"/>
       <c r="O23" s="16"/>
       <c r="P23" s="16"/>
       <c r="Q23" s="16"/>
@@ -30440,7 +30466,7 @@
       <c r="K24" s="17"/>
       <c r="L24" s="16"/>
       <c r="M24" s="16"/>
-      <c r="N24" s="21"/>
+      <c r="N24" s="20"/>
       <c r="O24" s="16"/>
       <c r="P24" s="16"/>
       <c r="Q24" s="16"/>
@@ -30471,11 +30497,9 @@
       <c r="I25" s="16"/>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
-      <c r="L25" s="28" t="s">
-        <v>120</v>
-      </c>
-      <c r="M25" s="28"/>
-      <c r="N25" s="21"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="20"/>
       <c r="O25" s="16"/>
       <c r="P25" s="16"/>
       <c r="Q25" s="16"/>
@@ -30494,6 +30518,12 @@
       <c r="AD25" s="16"/>
       <c r="AE25" s="16"/>
     </row>
+    <row r="27" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I27" s="29"/>
+    </row>
+    <row r="36" spans="9:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I36" s="26"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="N9" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>

</xml_diff>